<commit_message>
Update UI logic and Database for RFQ header and RFQ Item
</commit_message>
<xml_diff>
--- a/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
+++ b/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
@@ -5,24 +5,21 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E1639B1-D32A-4C4B-9570-0A703C6E45B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB9AF12-0672-4D6E-92B1-F47401BBD9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7C84AE3-DB05-4C95-9989-C46A2FC968FE}"/>
   </bookViews>
   <sheets>
     <sheet name="PRICED" sheetId="6" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">PRICED!$A$1:$AZ$52</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">PRICED!$1:$13</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>DESCRIPTION</t>
   </si>
@@ -90,9 +87,6 @@
     <t>QUANTITY</t>
   </si>
   <si>
-    <t>WEEKS</t>
-  </si>
-  <si>
     <t>SUB TOTAL</t>
   </si>
   <si>
@@ -120,15 +114,6 @@
     <t>: CG-0223-001000</t>
   </si>
   <si>
-    <t>Coolflow IGE concentrate</t>
-  </si>
-  <si>
-    <t>20L/Pail</t>
-  </si>
-  <si>
-    <t>Manufacturer :Hydratech</t>
-  </si>
-  <si>
     <t>SITI AMINAH</t>
   </si>
   <si>
@@ -136,9 +121,6 @@
   </si>
   <si>
     <t xml:space="preserve"> TOTAL PRICE</t>
-  </si>
-  <si>
-    <t>PAIL</t>
   </si>
   <si>
     <t>TOTAL PRICE (RM)</t>
@@ -182,7 +164,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -473,7 +455,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="77">
@@ -503,7 +485,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -824,23 +806,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="COVER"/>
-      <sheetName val="COMMERCIAL"/>
-      <sheetName val="TECHNICAL"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1199,7 +1164,6 @@
       <c r="AP1" s="2"/>
       <c r="AQ1" s="2"/>
       <c r="AR1" s="4" t="e">
-        <f>[1]COVER!AJ16</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -1242,7 +1206,6 @@
       <c r="AP2" s="2"/>
       <c r="AQ2" s="2"/>
       <c r="AR2" s="4" t="e">
-        <f>[1]COVER!AJ18</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -1639,7 +1602,7 @@
       <c r="B13" s="2"/>
       <c r="F13" s="5"/>
       <c r="G13" s="73" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H13" s="73"/>
       <c r="M13" s="2"/>
@@ -1714,7 +1677,7 @@
     </row>
     <row r="15" spans="1:44" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="6"/>
@@ -1723,7 +1686,7 @@
         <v>8</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H15" s="25"/>
       <c r="M15" s="2"/>
@@ -1767,7 +1730,7 @@
         <v>9</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H16" s="28"/>
       <c r="M16" s="2"/>
@@ -1811,7 +1774,7 @@
         <v>10</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H17" s="28"/>
       <c r="M17" s="2"/>
@@ -1855,7 +1818,7 @@
         <v>11</v>
       </c>
       <c r="G18" s="27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H18" s="28"/>
       <c r="M18" s="2"/>
@@ -1893,7 +1856,7 @@
     </row>
     <row r="19" spans="1:49" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="35" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B19" s="66"/>
       <c r="C19" s="9"/>
@@ -1902,7 +1865,7 @@
         <v>12</v>
       </c>
       <c r="G19" s="30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="31"/>
       <c r="M19" s="2"/>
@@ -2144,10 +2107,10 @@
         <v>15</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="H25" s="40" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="I25" s="50"/>
       <c r="J25" s="50"/>
@@ -2243,47 +2206,29 @@
       <c r="AW26" s="46"/>
     </row>
     <row r="27" spans="1:49" s="54" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="52">
-        <v>1</v>
-      </c>
-      <c r="B27" s="53" t="s">
-        <v>26</v>
-      </c>
+      <c r="A27" s="52"/>
+      <c r="B27" s="53"/>
       <c r="D27" s="55"/>
-      <c r="E27" s="52">
-        <v>12</v>
-      </c>
-      <c r="F27" s="56">
-        <v>50</v>
-      </c>
-      <c r="G27" s="57">
-        <v>1250</v>
-      </c>
+      <c r="E27" s="52"/>
+      <c r="F27" s="56"/>
+      <c r="G27" s="57"/>
       <c r="H27" s="57">
         <f>G27*F27</f>
-        <v>62500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:49" s="54" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="52"/>
-      <c r="B28" s="53" t="s">
-        <v>27</v>
-      </c>
+      <c r="B28" s="53"/>
       <c r="D28" s="55"/>
-      <c r="E28" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" s="52" t="s">
-        <v>32</v>
-      </c>
+      <c r="E28" s="52"/>
+      <c r="F28" s="52"/>
       <c r="G28" s="52"/>
       <c r="H28" s="52"/>
     </row>
     <row r="29" spans="1:49" s="54" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="52"/>
-      <c r="B29" s="53" t="s">
-        <v>28</v>
-      </c>
+      <c r="B29" s="53"/>
       <c r="D29" s="55"/>
       <c r="E29" s="58"/>
       <c r="F29" s="58"/>
@@ -2311,29 +2256,29 @@
     </row>
     <row r="32" spans="1:49" s="49" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F32" s="67" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G32" s="68"/>
       <c r="H32" s="64" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:11" s="49" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F33" s="67" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G33" s="68"/>
       <c r="H33" s="65" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:11" s="49" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F34" s="67" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G34" s="68"/>
       <c r="H34" s="64" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2347,7 +2292,7 @@
     </row>
     <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="37" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B38" s="37"/>
       <c r="C38" s="37"/>
@@ -2375,7 +2320,7 @@
     </row>
     <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="37" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B40" s="37"/>
       <c r="C40" s="37"/>
@@ -2390,7 +2335,7 @@
     </row>
     <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="37" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B41" s="37"/>
       <c r="C41" s="37"/>
@@ -2414,12 +2359,12 @@
     </row>
     <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="36" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2427,19 +2372,19 @@
     </row>
     <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F49" s="3"/>
     </row>
     <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F50" s="3"/>
     </row>
     <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F51" s="3"/>
     </row>

</xml_diff>

<commit_message>
Update RFQ if its the same quotecode
</commit_message>
<xml_diff>
--- a/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
+++ b/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\bin\Debug\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D544151-46DA-448E-AF40-9ECE249812FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F22DA87-32D7-4AB7-93B1-1E0FD1B0FA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7C84AE3-DB05-4C95-9989-C46A2FC968FE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="PRICED" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PRICED!$A$1:$AZ$49</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">PRICED!$1:$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PRICED!$A$1:$AI$93</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">PRICED!$1:$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -737,7 +737,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="3154680" y="160020"/>
+          <a:off x="3200400" y="160020"/>
           <a:ext cx="2316480" cy="807720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -773,15 +773,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>982980</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:colOff>883920</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>175260</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -796,7 +796,7 @@
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill>
+      <xdr:blipFill rotWithShape="1">
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
@@ -804,23 +804,19 @@
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="18689" t="10811" r="23544" b="48859"/>
+        <a:srcRect l="18267" t="9443" r="23153" b="48830"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1348740" y="8686800"/>
-          <a:ext cx="1043940" cy="899160"/>
+          <a:off x="1310640" y="7627620"/>
+          <a:ext cx="1059180" cy="929640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
             <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
@@ -1134,7 +1130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989ABBAC-D4A1-4D43-8C01-84364837E4AE}">
-  <dimension ref="A1:AZ175"/>
+  <dimension ref="A1:AY173"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" style="1" customWidth="1"/>
@@ -1142,9 +1138,9 @@
     <col min="3" max="3" width="4.109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="30.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.33203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="3" style="1" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="2.33203125" style="1" hidden="1" customWidth="1"/>
     <col min="11" max="18" width="9.109375" style="1" hidden="1" customWidth="1"/>
@@ -1153,18 +1149,11 @@
     <col min="25" max="25" width="0.6640625" style="1" hidden="1" customWidth="1"/>
     <col min="26" max="30" width="9.109375" style="1" hidden="1" customWidth="1"/>
     <col min="31" max="31" width="3" style="1" hidden="1" customWidth="1"/>
-    <col min="32" max="39" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="40" max="40" width="3.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="41" max="48" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="49" max="49" width="3" style="1" hidden="1" customWidth="1"/>
-    <col min="50" max="50" width="1.88671875" style="1" customWidth="1"/>
-    <col min="51" max="51" width="0.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="52" max="52" width="0.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="53" max="53" width="49.44140625" style="1" customWidth="1"/>
-    <col min="54" max="16384" width="9.109375" style="1"/>
+    <col min="32" max="35" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="36" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="2"/>
       <c r="F1" s="21" t="s">
         <v>2</v>
@@ -1194,19 +1183,8 @@
       <c r="AG1" s="2"/>
       <c r="AH1" s="2"/>
       <c r="AI1" s="2"/>
-      <c r="AJ1" s="2"/>
-      <c r="AK1" s="2"/>
-      <c r="AL1" s="2"/>
-      <c r="AM1" s="2"/>
-      <c r="AN1" s="2"/>
-      <c r="AO1" s="2"/>
-      <c r="AP1" s="2"/>
-      <c r="AQ1" s="2"/>
-      <c r="AR1" s="4" t="e">
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="2" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2"/>
       <c r="F2" s="22" t="s">
         <v>3</v>
@@ -1236,19 +1214,8 @@
       <c r="AG2" s="2"/>
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
-      <c r="AJ2" s="2"/>
-      <c r="AK2" s="2"/>
-      <c r="AL2" s="2"/>
-      <c r="AM2" s="2"/>
-      <c r="AN2" s="2"/>
-      <c r="AO2" s="2"/>
-      <c r="AP2" s="2"/>
-      <c r="AQ2" s="2"/>
-      <c r="AR2" s="4" t="e">
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="3" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
       <c r="F3" s="22" t="s">
         <v>4</v>
@@ -1278,17 +1245,8 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
-      <c r="AJ3" s="2"/>
-      <c r="AK3" s="2"/>
-      <c r="AL3" s="2"/>
-      <c r="AM3" s="2"/>
-      <c r="AN3" s="2"/>
-      <c r="AO3" s="2"/>
-      <c r="AP3" s="2"/>
-      <c r="AQ3" s="2"/>
-      <c r="AR3" s="4"/>
-    </row>
-    <row r="4" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="F4" s="22" t="s">
         <v>5</v>
@@ -1318,17 +1276,8 @@
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
-      <c r="AJ4" s="2"/>
-      <c r="AK4" s="2"/>
-      <c r="AL4" s="2"/>
-      <c r="AM4" s="2"/>
-      <c r="AN4" s="2"/>
-      <c r="AO4" s="2"/>
-      <c r="AP4" s="2"/>
-      <c r="AQ4" s="2"/>
-      <c r="AR4" s="4"/>
-    </row>
-    <row r="5" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="F5" s="22" t="s">
         <v>6</v>
@@ -1358,17 +1307,8 @@
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
-      <c r="AJ5" s="2"/>
-      <c r="AK5" s="2"/>
-      <c r="AL5" s="2"/>
-      <c r="AM5" s="2"/>
-      <c r="AN5" s="2"/>
-      <c r="AO5" s="2"/>
-      <c r="AP5" s="2"/>
-      <c r="AQ5" s="2"/>
-      <c r="AR5" s="4"/>
-    </row>
-    <row r="6" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
       <c r="F6" s="22" t="s">
         <v>7</v>
@@ -1398,17 +1338,8 @@
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
-      <c r="AJ6" s="2"/>
-      <c r="AK6" s="2"/>
-      <c r="AL6" s="2"/>
-      <c r="AM6" s="2"/>
-      <c r="AN6" s="2"/>
-      <c r="AO6" s="2"/>
-      <c r="AP6" s="2"/>
-      <c r="AQ6" s="2"/>
-      <c r="AR6" s="4"/>
-    </row>
-    <row r="7" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -1435,17 +1366,8 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
-      <c r="AJ7" s="2"/>
-      <c r="AK7" s="2"/>
-      <c r="AL7" s="2"/>
-      <c r="AM7" s="2"/>
-      <c r="AN7" s="2"/>
-      <c r="AO7" s="2"/>
-      <c r="AP7" s="2"/>
-      <c r="AQ7" s="2"/>
-      <c r="AR7" s="4"/>
-    </row>
-    <row r="8" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -1472,17 +1394,8 @@
       <c r="AG8" s="2"/>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
-      <c r="AJ8" s="2"/>
-      <c r="AK8" s="2"/>
-      <c r="AL8" s="2"/>
-      <c r="AM8" s="2"/>
-      <c r="AN8" s="2"/>
-      <c r="AO8" s="2"/>
-      <c r="AP8" s="2"/>
-      <c r="AQ8" s="2"/>
-      <c r="AR8" s="4"/>
-    </row>
-    <row r="9" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
@@ -1509,17 +1422,8 @@
       <c r="AG9" s="2"/>
       <c r="AH9" s="2"/>
       <c r="AI9" s="2"/>
-      <c r="AJ9" s="2"/>
-      <c r="AK9" s="2"/>
-      <c r="AL9" s="2"/>
-      <c r="AM9" s="2"/>
-      <c r="AN9" s="2"/>
-      <c r="AO9" s="2"/>
-      <c r="AP9" s="2"/>
-      <c r="AQ9" s="2"/>
-      <c r="AR9" s="4"/>
-    </row>
-    <row r="10" spans="1:44" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:35" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -1546,17 +1450,8 @@
       <c r="AG10" s="2"/>
       <c r="AH10" s="2"/>
       <c r="AI10" s="2"/>
-      <c r="AJ10" s="2"/>
-      <c r="AK10" s="2"/>
-      <c r="AL10" s="2"/>
-      <c r="AM10" s="2"/>
-      <c r="AN10" s="2"/>
-      <c r="AO10" s="2"/>
-      <c r="AP10" s="2"/>
-      <c r="AQ10" s="2"/>
-      <c r="AR10" s="4"/>
-    </row>
-    <row r="11" spans="1:44" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:35" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="58" t="s">
         <v>1</v>
       </c>
@@ -1590,17 +1485,8 @@
       <c r="AG11" s="2"/>
       <c r="AH11" s="2"/>
       <c r="AI11" s="2"/>
-      <c r="AJ11" s="2"/>
-      <c r="AK11" s="2"/>
-      <c r="AL11" s="2"/>
-      <c r="AM11" s="2"/>
-      <c r="AN11" s="2"/>
-      <c r="AO11" s="2"/>
-      <c r="AP11" s="2"/>
-      <c r="AQ11" s="2"/>
-      <c r="AR11" s="4"/>
-    </row>
-    <row r="12" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
@@ -1627,17 +1513,8 @@
       <c r="AG12" s="2"/>
       <c r="AH12" s="2"/>
       <c r="AI12" s="2"/>
-      <c r="AJ12" s="2"/>
-      <c r="AK12" s="2"/>
-      <c r="AL12" s="2"/>
-      <c r="AM12" s="2"/>
-      <c r="AN12" s="2"/>
-      <c r="AO12" s="2"/>
-      <c r="AP12" s="2"/>
-      <c r="AQ12" s="2"/>
-      <c r="AR12" s="4"/>
-    </row>
-    <row r="13" spans="1:44" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="F13" s="5"/>
       <c r="G13" s="61" t="s">
@@ -1667,17 +1544,8 @@
       <c r="AG13" s="2"/>
       <c r="AH13" s="2"/>
       <c r="AI13" s="2"/>
-      <c r="AJ13" s="2"/>
-      <c r="AK13" s="2"/>
-      <c r="AL13" s="2"/>
-      <c r="AM13" s="2"/>
-      <c r="AN13" s="2"/>
-      <c r="AO13" s="2"/>
-      <c r="AP13" s="2"/>
-      <c r="AQ13" s="2"/>
-      <c r="AR13" s="4"/>
-    </row>
-    <row r="14" spans="1:44" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:35" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -1704,17 +1572,8 @@
       <c r="AG14" s="2"/>
       <c r="AH14" s="2"/>
       <c r="AI14" s="2"/>
-      <c r="AJ14" s="2"/>
-      <c r="AK14" s="2"/>
-      <c r="AL14" s="2"/>
-      <c r="AM14" s="2"/>
-      <c r="AN14" s="2"/>
-      <c r="AO14" s="2"/>
-      <c r="AP14" s="2"/>
-      <c r="AQ14" s="2"/>
-      <c r="AR14" s="4"/>
-    </row>
-    <row r="15" spans="1:44" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:35" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>24</v>
       </c>
@@ -1753,17 +1612,8 @@
       <c r="AG15" s="2"/>
       <c r="AH15" s="2"/>
       <c r="AI15" s="2"/>
-      <c r="AJ15" s="2"/>
-      <c r="AK15" s="2"/>
-      <c r="AL15" s="2"/>
-      <c r="AM15" s="2"/>
-      <c r="AN15" s="2"/>
-      <c r="AO15" s="2"/>
-      <c r="AP15" s="2"/>
-      <c r="AQ15" s="2"/>
-      <c r="AR15" s="4"/>
-    </row>
-    <row r="16" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:35" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="34"/>
       <c r="B16" s="12"/>
       <c r="D16" s="8"/>
@@ -1797,17 +1647,8 @@
       <c r="AG16" s="2"/>
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
-      <c r="AJ16" s="2"/>
-      <c r="AK16" s="2"/>
-      <c r="AL16" s="2"/>
-      <c r="AM16" s="2"/>
-      <c r="AN16" s="2"/>
-      <c r="AO16" s="2"/>
-      <c r="AP16" s="2"/>
-      <c r="AQ16" s="2"/>
-      <c r="AR16" s="4"/>
-    </row>
-    <row r="17" spans="1:49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="34"/>
       <c r="B17" s="12"/>
       <c r="D17" s="8"/>
@@ -1841,17 +1682,8 @@
       <c r="AG17" s="2"/>
       <c r="AH17" s="2"/>
       <c r="AI17" s="2"/>
-      <c r="AJ17" s="2"/>
-      <c r="AK17" s="2"/>
-      <c r="AL17" s="2"/>
-      <c r="AM17" s="2"/>
-      <c r="AN17" s="2"/>
-      <c r="AO17" s="2"/>
-      <c r="AP17" s="2"/>
-      <c r="AQ17" s="2"/>
-      <c r="AR17" s="4"/>
-    </row>
-    <row r="18" spans="1:49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="54" t="s">
         <v>29</v>
       </c>
@@ -1889,17 +1721,8 @@
       <c r="AG18" s="2"/>
       <c r="AH18" s="2"/>
       <c r="AI18" s="2"/>
-      <c r="AJ18" s="2"/>
-      <c r="AK18" s="2"/>
-      <c r="AL18" s="2"/>
-      <c r="AM18" s="2"/>
-      <c r="AN18" s="2"/>
-      <c r="AO18" s="2"/>
-      <c r="AP18" s="2"/>
-      <c r="AQ18" s="2"/>
-      <c r="AR18" s="4"/>
-    </row>
-    <row r="19" spans="1:49" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:35" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="35" t="s">
         <v>28</v>
       </c>
@@ -1936,17 +1759,8 @@
       <c r="AG19" s="2"/>
       <c r="AH19" s="2"/>
       <c r="AI19" s="2"/>
-      <c r="AJ19" s="2"/>
-      <c r="AK19" s="2"/>
-      <c r="AL19" s="2"/>
-      <c r="AM19" s="2"/>
-      <c r="AN19" s="2"/>
-      <c r="AO19" s="2"/>
-      <c r="AP19" s="2"/>
-      <c r="AQ19" s="2"/>
-      <c r="AR19" s="4"/>
-    </row>
-    <row r="20" spans="1:49" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -1971,17 +1785,8 @@
       <c r="AG20" s="2"/>
       <c r="AH20" s="2"/>
       <c r="AI20" s="2"/>
-      <c r="AJ20" s="2"/>
-      <c r="AK20" s="2"/>
-      <c r="AL20" s="2"/>
-      <c r="AM20" s="2"/>
-      <c r="AN20" s="2"/>
-      <c r="AO20" s="2"/>
-      <c r="AP20" s="2"/>
-      <c r="AQ20" s="2"/>
-      <c r="AR20" s="4"/>
-    </row>
-    <row r="21" spans="1:49" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -2006,17 +1811,8 @@
       <c r="AG21" s="2"/>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
-      <c r="AJ21" s="2"/>
-      <c r="AK21" s="2"/>
-      <c r="AL21" s="2"/>
-      <c r="AM21" s="2"/>
-      <c r="AN21" s="2"/>
-      <c r="AO21" s="2"/>
-      <c r="AP21" s="2"/>
-      <c r="AQ21" s="2"/>
-      <c r="AR21" s="4"/>
-    </row>
-    <row r="22" spans="1:49" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -2041,17 +1837,8 @@
       <c r="AG22" s="2"/>
       <c r="AH22" s="2"/>
       <c r="AI22" s="2"/>
-      <c r="AJ22" s="2"/>
-      <c r="AK22" s="2"/>
-      <c r="AL22" s="2"/>
-      <c r="AM22" s="2"/>
-      <c r="AN22" s="2"/>
-      <c r="AO22" s="2"/>
-      <c r="AP22" s="2"/>
-      <c r="AQ22" s="2"/>
-      <c r="AR22" s="4"/>
-    </row>
-    <row r="23" spans="1:49" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="4"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -2076,17 +1863,8 @@
       <c r="AG23" s="2"/>
       <c r="AH23" s="2"/>
       <c r="AI23" s="2"/>
-      <c r="AJ23" s="2"/>
-      <c r="AK23" s="2"/>
-      <c r="AL23" s="2"/>
-      <c r="AM23" s="2"/>
-      <c r="AN23" s="2"/>
-      <c r="AO23" s="2"/>
-      <c r="AP23" s="2"/>
-      <c r="AQ23" s="2"/>
-      <c r="AR23" s="4"/>
-    </row>
-    <row r="24" spans="1:49" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:35" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="4"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -2121,22 +1899,8 @@
       <c r="AG24" s="2"/>
       <c r="AH24" s="2"/>
       <c r="AI24" s="2"/>
-      <c r="AJ24" s="2"/>
-      <c r="AK24" s="2"/>
-      <c r="AL24" s="2"/>
-      <c r="AM24" s="2"/>
-      <c r="AN24" s="2"/>
-      <c r="AO24" s="2"/>
-      <c r="AP24" s="2"/>
-      <c r="AQ24" s="2"/>
-      <c r="AR24" s="2"/>
-      <c r="AS24" s="2"/>
-      <c r="AT24" s="2"/>
-      <c r="AU24" s="2"/>
-      <c r="AV24" s="2"/>
-      <c r="AW24" s="2"/>
-    </row>
-    <row r="25" spans="1:49" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:35" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="38" t="s">
         <v>8</v>
       </c>
@@ -2184,22 +1948,8 @@
       <c r="AG25" s="45"/>
       <c r="AH25" s="45"/>
       <c r="AI25" s="45"/>
-      <c r="AJ25" s="45"/>
-      <c r="AK25" s="45"/>
-      <c r="AL25" s="45"/>
-      <c r="AM25" s="45"/>
-      <c r="AN25" s="45"/>
-      <c r="AO25" s="45"/>
-      <c r="AP25" s="45"/>
-      <c r="AQ25" s="45"/>
-      <c r="AR25" s="45"/>
-      <c r="AS25" s="45"/>
-      <c r="AT25" s="45"/>
-      <c r="AU25" s="45"/>
-      <c r="AV25" s="45"/>
-      <c r="AW25" s="45"/>
-    </row>
-    <row r="26" spans="1:49" s="44" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="40"/>
       <c r="B26" s="71"/>
       <c r="C26" s="72"/>
@@ -2235,22 +1985,8 @@
       <c r="AG26" s="42"/>
       <c r="AH26" s="42"/>
       <c r="AI26" s="42"/>
-      <c r="AJ26" s="42"/>
-      <c r="AK26" s="42"/>
-      <c r="AL26" s="42"/>
-      <c r="AM26" s="42"/>
-      <c r="AN26" s="42"/>
-      <c r="AO26" s="42"/>
-      <c r="AP26" s="42"/>
-      <c r="AQ26" s="42"/>
-      <c r="AR26" s="42"/>
-      <c r="AS26" s="42"/>
-      <c r="AT26" s="42"/>
-      <c r="AU26" s="42"/>
-      <c r="AV26" s="42"/>
-      <c r="AW26" s="42"/>
-    </row>
-    <row r="27" spans="1:49" s="48" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    </row>
+    <row r="27" spans="1:35" s="48" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="47" t="s">
         <v>42</v>
       </c>
@@ -2272,7 +2008,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:49" s="44" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="43"/>
       <c r="B28" s="68"/>
       <c r="C28" s="69"/>
@@ -2282,7 +2018,7 @@
       <c r="G28" s="43"/>
       <c r="H28" s="43"/>
     </row>
-    <row r="29" spans="1:49" s="44" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:35" s="44" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F29" s="55" t="s">
         <v>11</v>
       </c>
@@ -2291,7 +2027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:49" s="44" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:35" s="44" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F30" s="55" t="s">
         <v>12</v>
       </c>
@@ -2300,7 +2036,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:49" s="44" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:35" s="44" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F31" s="55" t="s">
         <v>19</v>
       </c>
@@ -2309,18 +2045,40 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:49" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
     </row>
-    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-    </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
+    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+      <c r="J33"/>
+      <c r="K33"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="37"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34"/>
+      <c r="K34"/>
     </row>
     <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="37" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B35" s="37"/>
       <c r="C35" s="37"/>
@@ -2334,101 +2092,90 @@
       <c r="K35"/>
     </row>
     <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="37"/>
-      <c r="B36" s="37"/>
-      <c r="C36" s="37"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
+      <c r="A36" s="74" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="74"/>
+      <c r="C36" s="74"/>
+      <c r="D36" s="74"/>
+      <c r="E36" s="74"/>
+      <c r="F36" s="74"/>
       <c r="G36"/>
       <c r="H36"/>
       <c r="I36"/>
       <c r="J36"/>
       <c r="K36"/>
     </row>
-    <row r="37" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-      <c r="J37"/>
-      <c r="K37"/>
-    </row>
-    <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="74" t="s">
-        <v>48</v>
-      </c>
-      <c r="B38" s="74"/>
-      <c r="C38" s="74"/>
-      <c r="D38" s="74"/>
-      <c r="E38" s="74"/>
-      <c r="F38" s="74"/>
-      <c r="G38"/>
-      <c r="H38"/>
-      <c r="I38"/>
-      <c r="J38"/>
-      <c r="K38"/>
+    <row r="37" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3"/>
     </row>
     <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
     </row>
     <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="3"/>
-    </row>
-    <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+      <c r="A40" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="36" t="s">
+    <row r="42" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="36" t="s">
         <v>17</v>
       </c>
     </row>
+    <row r="43" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="3"/>
+    </row>
     <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
+      <c r="A45" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="3"/>
     </row>
     <row r="46" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F46" s="3"/>
     </row>
     <row r="47" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" s="3"/>
+      <c r="A47" s="3"/>
     </row>
     <row r="48" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F48" s="3"/>
+      <c r="A48" s="3"/>
     </row>
     <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="15"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="H49" s="11"/>
+    </row>
+    <row r="50" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
-    </row>
-    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="14"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="16"/>
+    </row>
+    <row r="51" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
-      <c r="B51" s="15"/>
+      <c r="B51" s="14"/>
       <c r="C51" s="2"/>
       <c r="D51" s="15"/>
       <c r="E51" s="15"/>
-      <c r="H51" s="11"/>
     </row>
     <row r="52" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
@@ -2436,9 +2183,6 @@
       <c r="C52" s="2"/>
       <c r="D52" s="15"/>
       <c r="E52" s="15"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="16"/>
     </row>
     <row r="53" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
@@ -2474,114 +2218,100 @@
       <c r="C57" s="2"/>
       <c r="D57" s="15"/>
       <c r="E57" s="15"/>
+      <c r="H57" s="11"/>
     </row>
     <row r="58" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
+      <c r="B58" s="57"/>
+      <c r="C58" s="57"/>
+      <c r="D58" s="57"/>
+      <c r="E58" s="17"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="18"/>
     </row>
     <row r="59" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="H59" s="11"/>
+      <c r="H59" s="19"/>
     </row>
     <row r="60" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
-      <c r="B60" s="57"/>
-      <c r="C60" s="57"/>
-      <c r="D60" s="57"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="18"/>
-    </row>
-    <row r="61" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="3"/>
-      <c r="H61" s="19"/>
-    </row>
-    <row r="62" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="H62" s="19"/>
-    </row>
-    <row r="63" spans="1:8" ht="10.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B60" s="3"/>
+      <c r="H60" s="19"/>
+    </row>
+    <row r="61" spans="1:8" ht="10.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C65" s="2"/>
+    </row>
+    <row r="66" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C66" s="2"/>
+    </row>
     <row r="67" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C67" s="2"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
     </row>
     <row r="68" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C68" s="2"/>
-    </row>
-    <row r="69" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="2"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-    </row>
-    <row r="70" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="2"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-    </row>
-    <row r="71" spans="1:8" s="3" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-    </row>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+    </row>
+    <row r="69" spans="1:8" s="3" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1"/>
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+    </row>
+    <row r="70" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="72" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="73" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="74" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="75" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="1"/>
-      <c r="B97" s="1"/>
-      <c r="C97" s="1"/>
-      <c r="D97" s="1"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="1"/>
-      <c r="G97" s="1"/>
-      <c r="H97" s="1"/>
-    </row>
-    <row r="119" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="1"/>
-      <c r="B119" s="1"/>
-      <c r="C119" s="1"/>
-      <c r="D119" s="1"/>
-      <c r="E119" s="1"/>
-      <c r="F119" s="1"/>
-      <c r="G119" s="1"/>
-      <c r="H119" s="1"/>
-    </row>
-    <row r="141" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="1"/>
-      <c r="B141" s="1"/>
-      <c r="C141" s="1"/>
-      <c r="D141" s="1"/>
-      <c r="E141" s="1"/>
-      <c r="F141" s="1"/>
-      <c r="G141" s="1"/>
-      <c r="H141" s="1"/>
-    </row>
-    <row r="175" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M175" s="20"/>
+    <row r="95" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="1"/>
+    </row>
+    <row r="117" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="1"/>
+      <c r="B117" s="1"/>
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+      <c r="F117" s="1"/>
+      <c r="G117" s="1"/>
+      <c r="H117" s="1"/>
+    </row>
+    <row r="139" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="1"/>
+      <c r="B139" s="1"/>
+      <c r="C139" s="1"/>
+      <c r="D139" s="1"/>
+      <c r="E139" s="1"/>
+      <c r="F139" s="1"/>
+      <c r="G139" s="1"/>
+      <c r="H139" s="1"/>
+    </row>
+    <row r="173" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M173" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="F31:G31"/>
-    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B58:D58"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="B25:D25"/>
@@ -2590,7 +2320,7 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B26:D26"/>
-    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A36:F36"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.51181102362204722" right="0.39370078740157483" top="0.43307086614173229" bottom="0.62992125984251968" header="0.31496062992125984" footer="0.19685039370078741"/>

</xml_diff>

<commit_message>
Improve Excel/PDF generation, import robustness, installer
</commit_message>
<xml_diff>
--- a/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
+++ b/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F22DA87-32D7-4AB7-93B1-1E0FD1B0FA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7D4500-74E5-42FB-B48E-29FCB94883DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7C84AE3-DB05-4C95-9989-C46A2FC968FE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>DESCRIPTION</t>
   </si>
@@ -111,9 +111,6 @@
     <t>1. Cancellation of PO is subjected to penalty</t>
   </si>
   <si>
-    <t>TO :</t>
-  </si>
-  <si>
     <t>sub_total</t>
   </si>
   <si>
@@ -123,27 +120,6 @@
     <t>_discount</t>
   </si>
   <si>
-    <t>NO.</t>
-  </si>
-  <si>
-    <t>RFQ :</t>
-  </si>
-  <si>
-    <t>Date                :</t>
-  </si>
-  <si>
-    <t>Quotation No   :</t>
-  </si>
-  <si>
-    <t>Delivery Term  :</t>
-  </si>
-  <si>
-    <t>Payment  Term:</t>
-  </si>
-  <si>
-    <t>Validity           :</t>
-  </si>
-  <si>
     <t>client_name</t>
   </si>
   <si>
@@ -184,6 +160,27 @@
   </si>
   <si>
     <t>2. 10% of PO value will be charged upon late payment from the invoice date after 60 Days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quotation No   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery Term  </t>
+  </si>
+  <si>
+    <t>Payment  Term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validity           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO </t>
+  </si>
+  <si>
+    <t>RFQ NO.</t>
   </si>
 </sst>
 </file>
@@ -648,9 +645,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -673,6 +667,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -705,7 +702,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>53340</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1130,17 +1127,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989ABBAC-D4A1-4D43-8C01-84364837E4AE}">
-  <dimension ref="A1:AY173"/>
+  <dimension ref="A1:AI173"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="27" style="1" customWidth="1"/>
     <col min="3" max="3" width="4.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="3" style="1" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="2.33203125" style="1" hidden="1" customWidth="1"/>
     <col min="11" max="18" width="9.109375" style="1" hidden="1" customWidth="1"/>
@@ -1149,7 +1146,8 @@
     <col min="25" max="25" width="0.6640625" style="1" hidden="1" customWidth="1"/>
     <col min="26" max="30" width="9.109375" style="1" hidden="1" customWidth="1"/>
     <col min="31" max="31" width="3" style="1" hidden="1" customWidth="1"/>
-    <col min="32" max="35" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="32" max="34" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="1.6640625" style="1" hidden="1" customWidth="1"/>
     <col min="36" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
@@ -1575,18 +1573,18 @@
     </row>
     <row r="15" spans="1:35" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="7"/>
       <c r="F15" s="23" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H15" s="25"/>
       <c r="M15" s="2"/>
@@ -1618,10 +1616,10 @@
       <c r="B16" s="12"/>
       <c r="D16" s="8"/>
       <c r="F16" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G16" s="27" t="s">
         <v>31</v>
-      </c>
-      <c r="G16" s="27" t="s">
-        <v>39</v>
       </c>
       <c r="H16" s="28"/>
       <c r="M16" s="2"/>
@@ -1653,10 +1651,10 @@
       <c r="B17" s="12"/>
       <c r="D17" s="8"/>
       <c r="F17" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="27" t="s">
         <v>32</v>
-      </c>
-      <c r="G17" s="27" t="s">
-        <v>40</v>
       </c>
       <c r="H17" s="28"/>
       <c r="M17" s="2"/>
@@ -1685,17 +1683,17 @@
     </row>
     <row r="18" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="54" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D18" s="8"/>
       <c r="F18" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="27" t="s">
         <v>33</v>
-      </c>
-      <c r="G18" s="27" t="s">
-        <v>41</v>
       </c>
       <c r="H18" s="28"/>
       <c r="M18" s="2"/>
@@ -1723,17 +1721,15 @@
       <c r="AI18" s="2"/>
     </row>
     <row r="19" spans="1:35" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="35" t="s">
-        <v>28</v>
-      </c>
+      <c r="A19" s="35"/>
       <c r="B19" s="53"/>
       <c r="C19" s="9"/>
       <c r="D19" s="10"/>
       <c r="F19" s="29" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="G19" s="30" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H19" s="31"/>
       <c r="M19" s="2"/>
@@ -1951,9 +1947,9 @@
     </row>
     <row r="26" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="40"/>
-      <c r="B26" s="71"/>
-      <c r="C26" s="72"/>
-      <c r="D26" s="73"/>
+      <c r="B26" s="70"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="72"/>
       <c r="E26" s="41"/>
       <c r="F26" s="41"/>
       <c r="G26" s="41"/>
@@ -1988,31 +1984,31 @@
     </row>
     <row r="27" spans="1:35" s="48" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="47" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B27" s="65" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="66"/>
-      <c r="D27" s="67"/>
+        <v>35</v>
+      </c>
+      <c r="C27" s="74"/>
+      <c r="D27" s="66"/>
       <c r="E27" s="47" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G27" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H27" s="50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="43"/>
-      <c r="B28" s="68"/>
-      <c r="C28" s="69"/>
-      <c r="D28" s="70"/>
+      <c r="B28" s="67"/>
+      <c r="C28" s="68"/>
+      <c r="D28" s="69"/>
       <c r="E28" s="43"/>
       <c r="F28" s="43"/>
       <c r="G28" s="43"/>
@@ -2024,7 +2020,7 @@
       </c>
       <c r="G29" s="56"/>
       <c r="H29" s="51" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:35" s="44" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -2033,7 +2029,7 @@
       </c>
       <c r="G30" s="56"/>
       <c r="H30" s="52" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:35" s="44" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -2042,7 +2038,7 @@
       </c>
       <c r="G31" s="56"/>
       <c r="H31" s="51" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2092,14 +2088,14 @@
       <c r="K35"/>
     </row>
     <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="74" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="74"/>
-      <c r="C36" s="74"/>
-      <c r="D36" s="74"/>
-      <c r="E36" s="74"/>
-      <c r="F36" s="74"/>
+      <c r="A36" s="73" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="73"/>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
       <c r="G36"/>
       <c r="H36"/>
       <c r="I36"/>

</xml_diff>

<commit_message>
Update to v2.1: Excel border fix, dedup import, UI tweaks
- Bump project version to 2.1 and update deployment metadata
- Update Excel templates for improved page breaks and layout
- Refine Excel border logic: use subtotal row for page break borders
- Deduplicate repeated item descriptions on import to fix mid-item border bug
- Change currency dropdown: "$" → "USD", auto-select for PFLNG1
- Require "Validity" field before file generation
- Standardize temp/output file naming with hyphens
- "Generate Both Excel" now only generates PRICED version
- Default Excel file name now uses company/client codes
- UI anchoring/layout improvements for better resizing
- Code cleanup and improved comments throughout
</commit_message>
<xml_diff>
--- a/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
+++ b/RFQ Generator Beta Version/Templates/CG TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7D4500-74E5-42FB-B48E-29FCB94883DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6D0A33-E9C0-46C9-A62E-717B267305EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7C84AE3-DB05-4C95-9989-C46A2FC968FE}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PRICED" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PRICED!$A$1:$AI$93</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PRICED!$A$1:$AK$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">PRICED!$1:$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>DESCRIPTION</t>
   </si>
@@ -72,115 +72,118 @@
     <t>QUANTITY</t>
   </si>
   <si>
+    <t>Sales Executive</t>
+  </si>
+  <si>
+    <t>Cekap Gagasan Sdn Bhd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regards, </t>
+  </si>
+  <si>
+    <t>COMMERCIAL</t>
+  </si>
+  <si>
+    <t>SITI AMINAH</t>
+  </si>
+  <si>
+    <t>SITI AMINAH BT MUHAMMAD</t>
+  </si>
+  <si>
+    <t>TOTAL PRICE (RM)</t>
+  </si>
+  <si>
+    <t>UNIT PRICE (RM)</t>
+  </si>
+  <si>
+    <t>Terms &amp; Conditions</t>
+  </si>
+  <si>
+    <t>1. Cancellation of PO is subjected to penalty</t>
+  </si>
+  <si>
+    <t>sub_total</t>
+  </si>
+  <si>
+    <t>total_price</t>
+  </si>
+  <si>
+    <t>client_name</t>
+  </si>
+  <si>
+    <t>rfq_code</t>
+  </si>
+  <si>
+    <t>_date</t>
+  </si>
+  <si>
+    <t>_validity</t>
+  </si>
+  <si>
+    <t>quote_code</t>
+  </si>
+  <si>
+    <t>delivery_term</t>
+  </si>
+  <si>
+    <t>30 days</t>
+  </si>
+  <si>
+    <t>_num</t>
+  </si>
+  <si>
+    <t>_desc</t>
+  </si>
+  <si>
+    <t>delivery_time</t>
+  </si>
+  <si>
+    <t>unit_price</t>
+  </si>
+  <si>
+    <t>_qty</t>
+  </si>
+  <si>
+    <t>2. 10% of PO value will be charged upon late payment from the invoice date after 60 Days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quotation No   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery Term  </t>
+  </si>
+  <si>
+    <t>Payment  Term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validity           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO </t>
+  </si>
+  <si>
+    <t>RFQ NO.</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
     <t>SUB TOTAL</t>
   </si>
   <si>
     <t>DISCOUNT</t>
   </si>
   <si>
-    <t>Sales Executive</t>
-  </si>
-  <si>
-    <t>Cekap Gagasan Sdn Bhd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regards, </t>
-  </si>
-  <si>
-    <t>COMMERCIAL</t>
-  </si>
-  <si>
-    <t>SITI AMINAH</t>
-  </si>
-  <si>
-    <t>SITI AMINAH BT MUHAMMAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TOTAL PRICE</t>
-  </si>
-  <si>
-    <t>TOTAL PRICE (RM)</t>
-  </si>
-  <si>
-    <t>UNIT PRICE (RM)</t>
-  </si>
-  <si>
-    <t>Terms &amp; Conditions</t>
-  </si>
-  <si>
-    <t>1. Cancellation of PO is subjected to penalty</t>
-  </si>
-  <si>
-    <t>sub_total</t>
-  </si>
-  <si>
-    <t>total_price</t>
-  </si>
-  <si>
     <t>_discount</t>
   </si>
   <si>
-    <t>client_name</t>
-  </si>
-  <si>
-    <t>rfq_code</t>
-  </si>
-  <si>
-    <t>_date</t>
-  </si>
-  <si>
-    <t>_validity</t>
-  </si>
-  <si>
-    <t>quote_code</t>
-  </si>
-  <si>
-    <t>delivery_term</t>
-  </si>
-  <si>
-    <t>30 days</t>
-  </si>
-  <si>
-    <t>_num</t>
-  </si>
-  <si>
-    <t>_desc</t>
-  </si>
-  <si>
-    <t>delivery_time</t>
-  </si>
-  <si>
-    <t>unit_price</t>
+    <t>TOTALPRICE</t>
   </si>
   <si>
     <t>summary_total_price</t>
-  </si>
-  <si>
-    <t>_qty</t>
-  </si>
-  <si>
-    <t>2. 10% of PO value will be charged upon late payment from the invoice date after 60 Days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date                </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quotation No   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delivery Term  </t>
-  </si>
-  <si>
-    <t>Payment  Term</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validity           </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO </t>
-  </si>
-  <si>
-    <t>RFQ NO.</t>
   </si>
 </sst>
 </file>
@@ -482,7 +485,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -553,12 +556,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -594,30 +591,81 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="12" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -633,44 +681,38 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -695,13 +737,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>655320</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>53340</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -769,70 +811,50 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>883920</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1005840</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>130973</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>184310</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2202" name="Picture 4">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A412712-592D-F923-9C23-161FA77139D0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76D8E04F-860F-0154-79C7-65765D959B87}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="18267" t="9443" r="23153" b="48830"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="1310640" y="7627620"/>
-          <a:ext cx="1059180" cy="929640"/>
+          <a:off x="1722120" y="7299960"/>
+          <a:ext cx="976793" cy="931070"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1127,39 +1149,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989ABBAC-D4A1-4D43-8C01-84364837E4AE}">
-  <dimension ref="A1:AI173"/>
+  <dimension ref="A1:AK174"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="27" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="3" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="2.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="11" max="18" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="0.5546875" style="1" hidden="1" customWidth="1"/>
-    <col min="20" max="24" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="0.6640625" style="1" hidden="1" customWidth="1"/>
-    <col min="26" max="30" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="3" style="1" hidden="1" customWidth="1"/>
-    <col min="32" max="34" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="1.6640625" style="1" hidden="1" customWidth="1"/>
-    <col min="36" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="1" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27" style="1" customWidth="1"/>
+    <col min="4" max="4" width="4.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="1.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3" style="1" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="2.33203125" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="20" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="0.5546875" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="26" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="0.6640625" style="1" hidden="1" customWidth="1"/>
+    <col min="28" max="32" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="3" style="1" hidden="1" customWidth="1"/>
+    <col min="34" max="36" width="9.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="1.6640625" style="1" hidden="1" customWidth="1"/>
+    <col min="38" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="2"/>
-      <c r="F1" s="21" t="s">
+    <row r="1" spans="1:37" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="2"/>
+      <c r="G1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="4"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="4"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
@@ -1181,16 +1204,17 @@
       <c r="AG1" s="2"/>
       <c r="AH1" s="2"/>
       <c r="AI1" s="2"/>
-    </row>
-    <row r="2" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-      <c r="F2" s="22" t="s">
+      <c r="AJ1" s="2"/>
+      <c r="AK1" s="2"/>
+    </row>
+    <row r="2" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="2"/>
+      <c r="G2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="22"/>
-      <c r="H2" s="4"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="4"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -1212,16 +1236,17 @@
       <c r="AG2" s="2"/>
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
-    </row>
-    <row r="3" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="F3" s="22" t="s">
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+    </row>
+    <row r="3" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="2"/>
+      <c r="G3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="22"/>
-      <c r="H3" s="4"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="4"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -1243,16 +1268,17 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
-    </row>
-    <row r="4" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="F4" s="22" t="s">
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2"/>
+    </row>
+    <row r="4" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="2"/>
+      <c r="G4" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="4"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="4"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -1274,16 +1300,17 @@
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
-    </row>
-    <row r="5" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="F5" s="22" t="s">
+      <c r="AJ4" s="2"/>
+      <c r="AK4" s="2"/>
+    </row>
+    <row r="5" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+      <c r="G5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="22"/>
-      <c r="H5" s="4"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="4"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -1305,16 +1332,17 @@
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
-    </row>
-    <row r="6" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-      <c r="F6" s="22" t="s">
+      <c r="AJ5" s="2"/>
+      <c r="AK5" s="2"/>
+    </row>
+    <row r="6" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="2"/>
+      <c r="G6" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="22"/>
-      <c r="H6" s="4"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="4"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -1336,13 +1364,14 @@
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
-    </row>
-    <row r="7" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="F7" s="5"/>
+      <c r="AJ6" s="2"/>
+      <c r="AK6" s="2"/>
+    </row>
+    <row r="7" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="2"/>
       <c r="G7" s="5"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
@@ -1364,13 +1393,14 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
-    </row>
-    <row r="8" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="F8" s="5"/>
+      <c r="AJ7" s="2"/>
+      <c r="AK7" s="2"/>
+    </row>
+    <row r="8" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="2"/>
       <c r="G8" s="5"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
@@ -1392,13 +1422,14 @@
       <c r="AG8" s="2"/>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
-    </row>
-    <row r="9" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-      <c r="F9" s="5"/>
+      <c r="AJ8" s="2"/>
+      <c r="AK8" s="2"/>
+    </row>
+    <row r="9" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="2"/>
       <c r="G9" s="5"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
@@ -1420,13 +1451,14 @@
       <c r="AG9" s="2"/>
       <c r="AH9" s="2"/>
       <c r="AI9" s="2"/>
-    </row>
-    <row r="10" spans="1:35" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="2"/>
-      <c r="F10" s="5"/>
+      <c r="AJ9" s="2"/>
+      <c r="AK9" s="2"/>
+    </row>
+    <row r="10" spans="1:37" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="2"/>
       <c r="G10" s="5"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
@@ -1448,20 +1480,22 @@
       <c r="AG10" s="2"/>
       <c r="AH10" s="2"/>
       <c r="AI10" s="2"/>
-    </row>
-    <row r="11" spans="1:35" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="58" t="s">
+      <c r="AJ10" s="2"/>
+      <c r="AK10" s="2"/>
+    </row>
+    <row r="11" spans="1:37" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="60"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+      <c r="B11" s="74"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="75"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
@@ -1483,13 +1517,14 @@
       <c r="AG11" s="2"/>
       <c r="AH11" s="2"/>
       <c r="AI11" s="2"/>
-    </row>
-    <row r="12" spans="1:35" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="F12" s="5"/>
+      <c r="AJ11" s="2"/>
+      <c r="AK11" s="2"/>
+    </row>
+    <row r="12" spans="1:37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="2"/>
       <c r="G12" s="5"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
@@ -1511,16 +1546,17 @@
       <c r="AG12" s="2"/>
       <c r="AH12" s="2"/>
       <c r="AI12" s="2"/>
-    </row>
-    <row r="13" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="H13" s="61"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
+      <c r="AJ12" s="2"/>
+      <c r="AK12" s="2"/>
+    </row>
+    <row r="13" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="76" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" s="76"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
@@ -1542,13 +1578,14 @@
       <c r="AG13" s="2"/>
       <c r="AH13" s="2"/>
       <c r="AI13" s="2"/>
-    </row>
-    <row r="14" spans="1:35" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="F14" s="5"/>
+      <c r="AJ13" s="2"/>
+      <c r="AK13" s="2"/>
+    </row>
+    <row r="14" spans="1:37" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="2"/>
       <c r="G14" s="5"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
@@ -1570,25 +1607,31 @@
       <c r="AG14" s="2"/>
       <c r="AH14" s="2"/>
       <c r="AI14" s="2"/>
-    </row>
-    <row r="15" spans="1:35" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="7"/>
-      <c r="F15" s="23" t="s">
+      <c r="AJ14" s="2"/>
+      <c r="AK14" s="2"/>
+    </row>
+    <row r="15" spans="1:37" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="G15" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="25"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
+      <c r="B15" s="52" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="52" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="7"/>
+      <c r="G15" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" s="25"/>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
@@ -1610,20 +1653,24 @@
       <c r="AG15" s="2"/>
       <c r="AH15" s="2"/>
       <c r="AI15" s="2"/>
-    </row>
-    <row r="16" spans="1:35" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
+      <c r="AJ15" s="2"/>
+      <c r="AK15" s="2"/>
+    </row>
+    <row r="16" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="32"/>
       <c r="B16" s="12"/>
-      <c r="D16" s="8"/>
-      <c r="F16" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="G16" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="H16" s="28"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
+      <c r="C16" s="12"/>
+      <c r="E16" s="8"/>
+      <c r="G16" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="28"/>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
@@ -1645,20 +1692,24 @@
       <c r="AG16" s="2"/>
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
-    </row>
-    <row r="17" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="34"/>
+      <c r="AJ16" s="2"/>
+      <c r="AK16" s="2"/>
+    </row>
+    <row r="17" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="32"/>
       <c r="B17" s="12"/>
-      <c r="D17" s="8"/>
-      <c r="F17" s="26" t="s">
+      <c r="C17" s="12"/>
+      <c r="E17" s="8"/>
+      <c r="G17" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" s="28"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
+      <c r="I17" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" s="28"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
@@ -1680,24 +1731,30 @@
       <c r="AG17" s="2"/>
       <c r="AH17" s="2"/>
       <c r="AI17" s="2"/>
-    </row>
-    <row r="18" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="8"/>
-      <c r="F18" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="G18" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="H18" s="28"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
+      <c r="AJ17" s="2"/>
+      <c r="AK17" s="2"/>
+    </row>
+    <row r="18" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="50" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="G18" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="28"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
@@ -1719,21 +1776,25 @@
       <c r="AG18" s="2"/>
       <c r="AH18" s="2"/>
       <c r="AI18" s="2"/>
-    </row>
-    <row r="19" spans="1:35" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="35"/>
-      <c r="B19" s="53"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10"/>
-      <c r="F19" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="H19" s="31"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
+      <c r="AJ18" s="2"/>
+      <c r="AK18" s="2"/>
+    </row>
+    <row r="19" spans="1:37" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="33"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="10"/>
+      <c r="G19" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="I19" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="J19" s="31"/>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
@@ -1755,11 +1816,11 @@
       <c r="AG19" s="2"/>
       <c r="AH19" s="2"/>
       <c r="AI19" s="2"/>
-    </row>
-    <row r="20" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
+      <c r="AJ19" s="2"/>
+      <c r="AK19" s="2"/>
+    </row>
+    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
@@ -1781,11 +1842,11 @@
       <c r="AG20" s="2"/>
       <c r="AH20" s="2"/>
       <c r="AI20" s="2"/>
-    </row>
-    <row r="21" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
+      <c r="AJ20" s="2"/>
+      <c r="AK20" s="2"/>
+    </row>
+    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
@@ -1807,11 +1868,11 @@
       <c r="AG21" s="2"/>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
-    </row>
-    <row r="22" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
+      <c r="AJ21" s="2"/>
+      <c r="AK21" s="2"/>
+    </row>
+    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
@@ -1833,11 +1894,11 @@
       <c r="AG22" s="2"/>
       <c r="AH22" s="2"/>
       <c r="AI22" s="2"/>
-    </row>
-    <row r="23" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="4"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
+      <c r="AJ22" s="2"/>
+      <c r="AK22" s="2"/>
+    </row>
+    <row r="23" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="4"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
@@ -1859,10 +1920,11 @@
       <c r="AG23" s="2"/>
       <c r="AH23" s="2"/>
       <c r="AI23" s="2"/>
-    </row>
-    <row r="24" spans="1:35" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="4"/>
-      <c r="C24" s="2"/>
+      <c r="AJ23" s="2"/>
+      <c r="AK23" s="2"/>
+    </row>
+    <row r="24" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="4"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -1895,175 +1957,189 @@
       <c r="AG24" s="2"/>
       <c r="AH24" s="2"/>
       <c r="AI24" s="2"/>
-    </row>
-    <row r="25" spans="1:35" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="38" t="s">
+      <c r="AJ24" s="2"/>
+      <c r="AK24" s="2"/>
+    </row>
+    <row r="25" spans="1:37" s="44" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="62" t="s">
+      <c r="B25" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="C25" s="63"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="38" t="s">
+      <c r="C25" s="86"/>
+      <c r="D25" s="86"/>
+      <c r="E25" s="79"/>
+      <c r="F25" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="F25" s="38" t="s">
+      <c r="G25" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="G25" s="39" t="s">
+      <c r="H25" s="79"/>
+      <c r="I25" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J25" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="43"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="43"/>
+      <c r="N25" s="43"/>
+      <c r="O25" s="43"/>
+      <c r="P25" s="43"/>
+      <c r="Q25" s="43"/>
+      <c r="R25" s="43"/>
+      <c r="S25" s="43"/>
+      <c r="T25" s="43"/>
+      <c r="U25" s="43"/>
+      <c r="V25" s="43"/>
+      <c r="W25" s="43"/>
+      <c r="X25" s="43"/>
+      <c r="Y25" s="43"/>
+      <c r="Z25" s="43"/>
+      <c r="AA25" s="43"/>
+      <c r="AB25" s="43"/>
+      <c r="AC25" s="43"/>
+      <c r="AD25" s="43"/>
+      <c r="AE25" s="43"/>
+      <c r="AF25" s="43"/>
+      <c r="AG25" s="43"/>
+      <c r="AH25" s="43"/>
+      <c r="AI25" s="43"/>
+      <c r="AJ25" s="43"/>
+      <c r="AK25" s="43"/>
+    </row>
+    <row r="26" spans="1:37" s="42" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="38"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="80"/>
+      <c r="H26" s="81"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="40"/>
+      <c r="M26" s="40"/>
+      <c r="N26" s="40"/>
+      <c r="O26" s="40"/>
+      <c r="P26" s="40"/>
+      <c r="Q26" s="40"/>
+      <c r="R26" s="40"/>
+      <c r="S26" s="40"/>
+      <c r="T26" s="40"/>
+      <c r="U26" s="40"/>
+      <c r="V26" s="40"/>
+      <c r="W26" s="40"/>
+      <c r="X26" s="40"/>
+      <c r="Y26" s="40"/>
+      <c r="Z26" s="40"/>
+      <c r="AA26" s="40"/>
+      <c r="AB26" s="40"/>
+      <c r="AC26" s="40"/>
+      <c r="AD26" s="40"/>
+      <c r="AE26" s="40"/>
+      <c r="AF26" s="40"/>
+      <c r="AG26" s="40"/>
+      <c r="AH26" s="40"/>
+      <c r="AI26" s="40"/>
+      <c r="AJ26" s="40"/>
+      <c r="AK26" s="40"/>
+    </row>
+    <row r="27" spans="1:37" s="46" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="68"/>
+      <c r="F27" s="45" t="s">
+        <v>32</v>
+      </c>
+      <c r="G27" s="82" t="s">
+        <v>34</v>
+      </c>
+      <c r="H27" s="83"/>
+      <c r="I27" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="J27" s="47" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:37" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="41"/>
+      <c r="B28" s="69"/>
+      <c r="C28" s="70"/>
+      <c r="D28" s="70"/>
+      <c r="E28" s="71"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="85"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="41"/>
+    </row>
+    <row r="29" spans="1:37" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B29" s="55"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
+      <c r="G29" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="H29" s="58"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="H25" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="I25" s="45"/>
-      <c r="J25" s="45"/>
-      <c r="K25" s="45"/>
-      <c r="L25" s="45"/>
-      <c r="M25" s="45"/>
-      <c r="N25" s="45"/>
-      <c r="O25" s="45"/>
-      <c r="P25" s="45"/>
-      <c r="Q25" s="45"/>
-      <c r="R25" s="45"/>
-      <c r="S25" s="45"/>
-      <c r="T25" s="45"/>
-      <c r="U25" s="45"/>
-      <c r="V25" s="45"/>
-      <c r="W25" s="45"/>
-      <c r="X25" s="45"/>
-      <c r="Y25" s="45"/>
-      <c r="Z25" s="45"/>
-      <c r="AA25" s="45"/>
-      <c r="AB25" s="45"/>
-      <c r="AC25" s="45"/>
-      <c r="AD25" s="45"/>
-      <c r="AE25" s="45"/>
-      <c r="AF25" s="45"/>
-      <c r="AG25" s="45"/>
-      <c r="AH25" s="45"/>
-      <c r="AI25" s="45"/>
-    </row>
-    <row r="26" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="40"/>
-      <c r="B26" s="70"/>
-      <c r="C26" s="71"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="41"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="42"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
-      <c r="O26" s="42"/>
-      <c r="P26" s="42"/>
-      <c r="Q26" s="42"/>
-      <c r="R26" s="42"/>
-      <c r="S26" s="42"/>
-      <c r="T26" s="42"/>
-      <c r="U26" s="42"/>
-      <c r="V26" s="42"/>
-      <c r="W26" s="42"/>
-      <c r="X26" s="42"/>
-      <c r="Y26" s="42"/>
-      <c r="Z26" s="42"/>
-      <c r="AA26" s="42"/>
-      <c r="AB26" s="42"/>
-      <c r="AC26" s="42"/>
-      <c r="AD26" s="42"/>
-      <c r="AE26" s="42"/>
-      <c r="AF26" s="42"/>
-      <c r="AG26" s="42"/>
-      <c r="AH26" s="42"/>
-      <c r="AI26" s="42"/>
-    </row>
-    <row r="27" spans="1:35" s="48" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" s="65" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="F27" s="49" t="s">
-        <v>39</v>
-      </c>
-      <c r="G27" s="50" t="s">
-        <v>37</v>
-      </c>
-      <c r="H27" s="50" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:35" s="44" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="43"/>
-      <c r="B28" s="67"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="69"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-    </row>
-    <row r="29" spans="1:35" s="44" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F29" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="G29" s="56"/>
-      <c r="H29" s="51" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:35" s="44" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F30" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="G30" s="56"/>
-      <c r="H30" s="52" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:35" s="44" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F31" s="55" t="s">
+    </row>
+    <row r="30" spans="1:37" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="55"/>
+      <c r="G30" s="57" t="s">
+        <v>45</v>
+      </c>
+      <c r="H30" s="58"/>
+      <c r="I30" s="59"/>
+      <c r="J30" s="56" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B31" s="55"/>
+      <c r="C31" s="55"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="55"/>
+      <c r="G31" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="H31" s="61"/>
+      <c r="I31" s="62"/>
+      <c r="J31" s="87" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:37" s="42" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="33" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+    </row>
+    <row r="34" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="56"/>
-      <c r="H31" s="51" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="32" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-    </row>
-    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
-      <c r="I33"/>
-      <c r="J33"/>
-      <c r="K33"/>
-    </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="37"/>
-      <c r="B34" s="37"/>
-      <c r="C34" s="37"/>
-      <c r="D34"/>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
       <c r="E34"/>
       <c r="F34"/>
       <c r="G34"/>
@@ -2071,14 +2147,14 @@
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
-    </row>
-    <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35"/>
+      <c r="L34"/>
+      <c r="M34"/>
+    </row>
+    <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="35"/>
+      <c r="B35" s="35"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
       <c r="E35"/>
       <c r="F35"/>
       <c r="G35"/>
@@ -2086,237 +2162,299 @@
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
-    </row>
-    <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="73" t="s">
-        <v>40</v>
-      </c>
-      <c r="B36" s="73"/>
-      <c r="C36" s="73"/>
-      <c r="D36" s="73"/>
-      <c r="E36" s="73"/>
-      <c r="F36" s="73"/>
+      <c r="L35"/>
+      <c r="M35"/>
+    </row>
+    <row r="36" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="35"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="35"/>
+      <c r="E36"/>
+      <c r="F36"/>
       <c r="G36"/>
       <c r="H36"/>
       <c r="I36"/>
       <c r="J36"/>
       <c r="K36"/>
-    </row>
-    <row r="37" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="3"/>
-    </row>
-    <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L36"/>
+      <c r="M36"/>
+    </row>
+    <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="77"/>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="51"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+    </row>
+    <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
-    </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="3"/>
+    </row>
+    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
-    </row>
-    <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+      <c r="B39" s="3"/>
+    </row>
+    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+    </row>
+    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="34" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F44" s="3"/>
-    </row>
-    <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="34"/>
+    </row>
+    <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+    </row>
+    <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="46" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F46" s="3"/>
-    </row>
-    <row r="47" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-    </row>
-    <row r="48" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="3"/>
+    </row>
+    <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
-      <c r="H49" s="11"/>
-    </row>
-    <row r="50" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="3"/>
+    </row>
+    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="15"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="2"/>
       <c r="E50" s="15"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
-      <c r="H50" s="16"/>
-    </row>
-    <row r="51" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F50" s="15"/>
+      <c r="J50" s="11"/>
+    </row>
+    <row r="51" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="15"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="2"/>
       <c r="E51" s="15"/>
-    </row>
-    <row r="52" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F51" s="15"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="16"/>
+    </row>
+    <row r="52" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="15"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="2"/>
       <c r="E52" s="15"/>
-    </row>
-    <row r="53" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F52" s="15"/>
+    </row>
+    <row r="53" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="15"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="2"/>
       <c r="E53" s="15"/>
-    </row>
-    <row r="54" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F53" s="15"/>
+    </row>
+    <row r="54" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="15"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="2"/>
       <c r="E54" s="15"/>
-    </row>
-    <row r="55" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F54" s="15"/>
+    </row>
+    <row r="55" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="15"/>
+      <c r="B55" s="3"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="2"/>
       <c r="E55" s="15"/>
-    </row>
-    <row r="56" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="15"/>
+    </row>
+    <row r="56" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="15"/>
+      <c r="B56" s="3"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="2"/>
       <c r="E56" s="15"/>
-    </row>
-    <row r="57" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F56" s="15"/>
+    </row>
+    <row r="57" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="15"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="2"/>
       <c r="E57" s="15"/>
-      <c r="H57" s="11"/>
-    </row>
-    <row r="58" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F57" s="15"/>
+    </row>
+    <row r="58" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
-      <c r="B58" s="57"/>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="18"/>
-    </row>
-    <row r="59" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="3"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="15"/>
+      <c r="J58" s="11"/>
+    </row>
+    <row r="59" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
-      <c r="H59" s="19"/>
-    </row>
-    <row r="60" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="3"/>
+      <c r="C59" s="72"/>
+      <c r="D59" s="72"/>
+      <c r="E59" s="72"/>
+      <c r="F59" s="17"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="18"/>
+    </row>
+    <row r="60" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
-      <c r="H60" s="19"/>
-    </row>
-    <row r="61" spans="1:8" ht="10.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="2"/>
-    </row>
-    <row r="66" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="2"/>
-    </row>
-    <row r="67" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="2"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-    </row>
-    <row r="68" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="2"/>
-      <c r="F68" s="3"/>
+      <c r="J60" s="19"/>
+    </row>
+    <row r="61" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="J61" s="19"/>
+    </row>
+    <row r="62" spans="1:10" ht="10.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D66" s="2"/>
+    </row>
+    <row r="67" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D67" s="2"/>
+    </row>
+    <row r="68" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D68" s="2"/>
       <c r="G68" s="3"/>
-    </row>
-    <row r="69" spans="1:8" s="3" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="1"/>
-      <c r="B69" s="1"/>
-      <c r="C69" s="1"/>
-      <c r="D69" s="1"/>
-      <c r="E69" s="1"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-      <c r="H69" s="1"/>
-    </row>
-    <row r="70" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:8" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="1"/>
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-      <c r="D95" s="1"/>
-      <c r="E95" s="1"/>
-      <c r="F95" s="1"/>
-      <c r="G95" s="1"/>
-      <c r="H95" s="1"/>
-    </row>
-    <row r="117" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="1"/>
-      <c r="B117" s="1"/>
-      <c r="C117" s="1"/>
-      <c r="D117" s="1"/>
-      <c r="E117" s="1"/>
-      <c r="F117" s="1"/>
-      <c r="G117" s="1"/>
-      <c r="H117" s="1"/>
-    </row>
-    <row r="139" spans="1:8" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="1"/>
-      <c r="B139" s="1"/>
-      <c r="C139" s="1"/>
-      <c r="D139" s="1"/>
-      <c r="E139" s="1"/>
-      <c r="F139" s="1"/>
-      <c r="G139" s="1"/>
-      <c r="H139" s="1"/>
-    </row>
-    <row r="173" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M173" s="20"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+    </row>
+    <row r="69" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D69" s="2"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+    </row>
+    <row r="70" spans="1:10" s="3" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1"/>
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+    </row>
+    <row r="71" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:10" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
+      <c r="J96" s="1"/>
+    </row>
+    <row r="118" spans="1:10" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="1"/>
+      <c r="B118" s="1"/>
+      <c r="C118" s="1"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+      <c r="F118" s="1"/>
+      <c r="G118" s="1"/>
+      <c r="H118" s="1"/>
+      <c r="I118" s="1"/>
+      <c r="J118" s="1"/>
+    </row>
+    <row r="140" spans="1:10" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="1"/>
+      <c r="B140" s="1"/>
+      <c r="C140" s="1"/>
+      <c r="D140" s="1"/>
+      <c r="E140" s="1"/>
+      <c r="F140" s="1"/>
+      <c r="G140" s="1"/>
+      <c r="H140" s="1"/>
+      <c r="I140" s="1"/>
+      <c r="J140" s="1"/>
+    </row>
+    <row r="174" spans="15:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O174" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="A36:F36"/>
+  <mergeCells count="15">
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.51181102362204722" right="0.39370078740157483" top="0.43307086614173229" bottom="0.62992125984251968" header="0.31496062992125984" footer="0.19685039370078741"/>

</xml_diff>